<commit_message>
Read DeepBGC start coordinates as 0-based
DeepBGC writes 0-based, end-exclusive intervals in both its cluster table
(nucl_start) and its Pfam table (gene_start); the parser passed them through
as if 1-based, so every DeepBGC start was 1 bp early and a locus at the very
start of a contig began at position 0. Starts are now shifted by one; ends
were already right.

The validation was regenerated from the unchanged raw DeepBGC output with the
fixed parser (validation/reparse_deepbgc.py). DeepBGC-derived boundaries move
by 1 bp; no grouping, recovery status or per-genome result changes, and
BGC-QUAST still agrees on all 294 locus x set pairs. The example's
DeepBGC-only locus now starts at 1.
</commit_message>
<xml_diff>
--- a/validation/tables/supplementary_per_locus.xlsx
+++ b/validation/tables/supplementary_per_locus.xlsx
@@ -2006,7 +2006,7 @@
         </is>
       </c>
       <c r="P19" t="n">
-        <v>0.511</v>
+        <v>0.512</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
@@ -3556,7 +3556,7 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>0.394</v>
+        <v>0.395</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>

</xml_diff>